<commit_message>
fix: usar R32 oficial da plataforma e decidir mata-mata pelo placar Smart
- app.py: vencedor do mata-mata decidido pelo placar Smart (nao mais pela
  probabilidade de campeao); empate no tempo normal decide nos penaltis pelo
  favorito; adicionada disputa de 3o lugar (M103).
- gabarito_bolao_cli.xlsx: R32 substituido pelos confrontos reais da
  plataforma; R16-Final propagados pela arvore oficial FIFA 2026;
  classificacao de grupos, 8 melhores 3os e classificacao final atualizados.
</commit_message>
<xml_diff>
--- a/bolao_cli/gabarito_bolao_cli.xlsx
+++ b/bolao_cli/gabarito_bolao_cli.xlsx
@@ -3514,6 +3514,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
@@ -3537,28 +3538,28 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>1x2</t>
+          <t>0x2</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>NORMAL (d=0.08) -&gt; Canada</t>
+          <t>BIG (d=0.57) -&gt; Switzerland</t>
         </is>
       </c>
       <c r="G77" s="4" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="H77" s="4" t="n">
-        <v>1.05</v>
+        <v>1.58</v>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>27%</t>
         </is>
       </c>
     </row>
@@ -3573,33 +3574,33 @@
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.81) -&gt; Germany</t>
+          <t>NORMAL (d=0.45) -&gt; Ecuador</t>
         </is>
       </c>
       <c r="G78" s="10" t="n">
-        <v>1.88</v>
+        <v>1.19</v>
       </c>
       <c r="H78" s="10" t="n">
-        <v>1.08</v>
+        <v>0.74</v>
       </c>
       <c r="I78" s="10" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3615,7 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3629,18 +3630,18 @@
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>NORMAL (d=0.01) -&gt; Morocco</t>
+          <t>NORMAL (d=0.13) -&gt; Morocco</t>
         </is>
       </c>
       <c r="G79" s="4" t="n">
-        <v>0.92</v>
+        <v>0.99</v>
       </c>
       <c r="H79" s="4" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.12</v>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>32%</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3661,7 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
@@ -3670,18 +3671,18 @@
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.60) -&gt; Brazil</t>
+          <t>BIG (d=0.97) -&gt; Brazil</t>
         </is>
       </c>
       <c r="G80" s="10" t="n">
-        <v>1.66</v>
+        <v>1.52</v>
       </c>
       <c r="H80" s="10" t="n">
-        <v>1.06</v>
+        <v>0.55</v>
       </c>
       <c r="I80" s="10" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>28%</t>
         </is>
       </c>
     </row>
@@ -3701,28 +3702,28 @@
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>4x1</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>VERY BIG (d=1.41) -&gt; France</t>
+          <t>NORMAL (d=0.43) -&gt; France</t>
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>2.06</v>
+        <v>1.38</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>0.64</v>
+        <v>0.95</v>
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3738,7 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -3752,18 +3753,18 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>NORMAL (d=0.17) -&gt; Ecuador</t>
+          <t>NORMAL (d=0.23) -&gt; Germany</t>
         </is>
       </c>
       <c r="G82" s="4" t="n">
-        <v>0.99</v>
+        <v>1.78</v>
       </c>
       <c r="H82" s="4" t="n">
-        <v>0.83</v>
+        <v>1.56</v>
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -3783,28 +3784,28 @@
       </c>
       <c r="D83" s="13" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Scotland</t>
         </is>
       </c>
       <c r="E83" s="14" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="F83" s="13" t="inlineStr">
         <is>
-          <t>EMPATE -&gt; Ivory Coast</t>
+          <t>NORMAL (d=0.13) -&gt; Mexico</t>
         </is>
       </c>
       <c r="G83" s="13" t="n">
-        <v>0.89</v>
+        <v>1.09</v>
       </c>
       <c r="H83" s="13" t="n">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="I83" s="13" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -3834,11 +3835,11 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.52) -&gt; England</t>
+          <t>BIG (d=0.53) -&gt; England</t>
         </is>
       </c>
       <c r="G84" s="10" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="H84" s="10" t="n">
         <v>0.76</v>
@@ -3860,33 +3861,33 @@
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="E85" s="11" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>1x2</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=1.16) -&gt; Turkey</t>
+          <t>NORMAL (d=0.16) -&gt; Algeria</t>
         </is>
       </c>
       <c r="G85" s="10" t="n">
-        <v>2.03</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H85" s="10" t="n">
-        <v>0.86</v>
+        <v>1.1</v>
       </c>
       <c r="I85" s="10" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -3906,24 +3907,24 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>2x0</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>NORMAL (d=0.44) -&gt; Belgium</t>
+          <t>BIG (d=0.74) -&gt; Belgium</t>
         </is>
       </c>
       <c r="G86" s="4" t="n">
-        <v>1.59</v>
+        <v>1.66</v>
       </c>
       <c r="H86" s="4" t="n">
-        <v>1.15</v>
+        <v>0.92</v>
       </c>
       <c r="I86" s="4" t="inlineStr">
         <is>
@@ -3961,7 +3962,7 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
       <c r="H87" s="4" t="n">
         <v>1.02</v>
@@ -4002,7 +4003,7 @@
         </is>
       </c>
       <c r="G88" s="10" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="H88" s="10" t="n">
         <v>0.89</v>
@@ -4024,7 +4025,7 @@
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
@@ -4034,23 +4035,23 @@
       </c>
       <c r="E89" s="11" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.65) -&gt; Switzerland</t>
+          <t>EMPATE -&gt; Canada</t>
         </is>
       </c>
       <c r="G89" s="10" t="n">
-        <v>1.48</v>
+        <v>0.98</v>
       </c>
       <c r="H89" s="10" t="n">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="I89" s="10" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>35%</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4085,7 @@
         </is>
       </c>
       <c r="G90" s="13" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="H90" s="13" t="n">
         <v>0.54</v>
@@ -4111,7 +4112,7 @@
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="E91" s="11" t="inlineStr">
@@ -4121,18 +4122,18 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.98) -&gt; Portugal</t>
+          <t>BIG (d=1.03) -&gt; Portugal</t>
         </is>
       </c>
       <c r="G91" s="10" t="n">
-        <v>1.55</v>
+        <v>1.65</v>
       </c>
       <c r="H91" s="10" t="n">
-        <v>0.57</v>
+        <v>0.62</v>
       </c>
       <c r="I91" s="10" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>26%</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4163,7 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>NORMAL (d=0.05) -&gt; Australia</t>
+          <t>NORMAL (d=0.06) -&gt; Australia</t>
         </is>
       </c>
       <c r="G92" s="4" t="n">
@@ -4177,6 +4178,7 @@
         </is>
       </c>
     </row>
+    <row r="93"/>
     <row r="94">
       <c r="A94" s="9" t="n">
         <v>89</v>
@@ -4188,7 +4190,7 @@
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
@@ -4198,23 +4200,23 @@
       </c>
       <c r="E94" s="11" t="inlineStr">
         <is>
-          <t>0x2</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="F94" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.81) -&gt; France</t>
+          <t>EMPATE -&gt; France</t>
         </is>
       </c>
       <c r="G94" s="10" t="n">
-        <v>1.1</v>
+        <v>0.61</v>
       </c>
       <c r="H94" s="10" t="n">
-        <v>1.91</v>
+        <v>1.01</v>
       </c>
       <c r="I94" s="10" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
@@ -4229,7 +4231,7 @@
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
@@ -4239,23 +4241,23 @@
       </c>
       <c r="E95" s="11" t="inlineStr">
         <is>
-          <t>0x2</t>
+          <t>1x2</t>
         </is>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.52) -&gt; Morocco</t>
+          <t>NORMAL (d=0.25) -&gt; Morocco</t>
         </is>
       </c>
       <c r="G95" s="10" t="n">
-        <v>0.6</v>
+        <v>0.91</v>
       </c>
       <c r="H95" s="10" t="n">
-        <v>1.12</v>
+        <v>1.16</v>
       </c>
       <c r="I95" s="10" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>32%</t>
         </is>
       </c>
     </row>
@@ -4275,28 +4277,28 @@
       </c>
       <c r="D96" s="13" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E96" s="14" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>2x0</t>
         </is>
       </c>
       <c r="F96" s="13" t="inlineStr">
         <is>
-          <t>EMPATE -&gt; Brazil</t>
+          <t>BIG (d=0.78) -&gt; Brazil</t>
         </is>
       </c>
       <c r="G96" s="13" t="n">
-        <v>1.01</v>
+        <v>1.9</v>
       </c>
       <c r="H96" s="13" t="n">
-        <v>0.63</v>
+        <v>1.12</v>
       </c>
       <c r="I96" s="13" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>24%</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4313,7 @@
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
@@ -4326,18 +4328,18 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.68) -&gt; England</t>
+          <t>BIG (d=0.75) -&gt; England</t>
         </is>
       </c>
       <c r="G97" s="10" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="H97" s="10" t="n">
-        <v>1.29</v>
+        <v>1.37</v>
       </c>
       <c r="I97" s="10" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -4393,7 +4395,7 @@
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr">
@@ -4403,23 +4405,23 @@
       </c>
       <c r="E99" s="11" t="inlineStr">
         <is>
-          <t>0x2</t>
+          <t>1x2</t>
         </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.68) -&gt; Belgium</t>
+          <t>NORMAL (d=0.45) -&gt; Belgium</t>
         </is>
       </c>
       <c r="G99" s="10" t="n">
-        <v>1.2</v>
+        <v>1.14</v>
       </c>
       <c r="H99" s="10" t="n">
-        <v>1.88</v>
+        <v>1.59</v>
       </c>
       <c r="I99" s="10" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>27%</t>
         </is>
       </c>
     </row>
@@ -4449,11 +4451,11 @@
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.94) -&gt; Argentina</t>
+          <t>BIG (d=0.95) -&gt; Argentina</t>
         </is>
       </c>
       <c r="G100" s="10" t="n">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="H100" s="10" t="n">
         <v>0.44</v>
@@ -4475,7 +4477,7 @@
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
@@ -4490,14 +4492,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>BIG (d=0.76) -&gt; Portugal</t>
+          <t>BIG (d=1.01) -&gt; Portugal</t>
         </is>
       </c>
       <c r="G101" s="10" t="n">
-        <v>0.95</v>
+        <v>0.63</v>
       </c>
       <c r="H101" s="10" t="n">
-        <v>1.71</v>
+        <v>1.65</v>
       </c>
       <c r="I101" s="10" t="inlineStr">
         <is>
@@ -4505,6 +4507,7 @@
         </is>
       </c>
     </row>
+    <row r="102"/>
     <row r="103">
       <c r="A103" s="3" t="n">
         <v>97</v>
@@ -4531,11 +4534,11 @@
       </c>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>NORMAL (d=0.35) -&gt; France</t>
+          <t>NORMAL (d=0.34) -&gt; France</t>
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="H103" s="4" t="n">
         <v>0.8</v>
@@ -4579,7 +4582,7 @@
         <v>1.86</v>
       </c>
       <c r="H104" s="10" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="I104" s="10" t="inlineStr">
         <is>
@@ -4617,7 +4620,7 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="H105" s="4" t="n">
         <v>0.93</v>
@@ -4661,7 +4664,7 @@
         <v>1.09</v>
       </c>
       <c r="H106" s="4" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
@@ -4669,6 +4672,7 @@
         </is>
       </c>
     </row>
+    <row r="107"/>
     <row r="108">
       <c r="A108" s="3" t="n">
         <v>101</v>
@@ -4702,7 +4706,7 @@
         <v>1.25</v>
       </c>
       <c r="H108" s="4" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
@@ -4751,6 +4755,7 @@
         </is>
       </c>
     </row>
+    <row r="110"/>
     <row r="111">
       <c r="A111" s="3" t="n">
         <v>103</v>
@@ -4829,10 +4834,12 @@
       </c>
       <c r="I112" s="4" t="inlineStr">
         <is>
-          <t>32%</t>
-        </is>
-      </c>
-    </row>
+          <t>33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="113"/>
+    <row r="114"/>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
@@ -4888,6 +4895,7 @@
         </is>
       </c>
     </row>
+    <row r="120"/>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
@@ -4920,12 +4928,12 @@
       </c>
       <c r="C123" s="15" t="inlineStr">
         <is>
-          <t>1o: Switzerland</t>
+          <t>1o: Canada</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2o: Canada</t>
+          <t>2o: Switzerland</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4962,7 @@
       </c>
       <c r="C125" s="15" t="inlineStr">
         <is>
-          <t>1o: Turkey</t>
+          <t>1o: Paraguay</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4971,12 +4979,12 @@
       </c>
       <c r="C126" s="15" t="inlineStr">
         <is>
-          <t>1o: Germany</t>
+          <t>1o: Ecuador</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2o: Ecuador</t>
+          <t>2o: Germany</t>
         </is>
       </c>
     </row>
@@ -4988,12 +4996,12 @@
       </c>
       <c r="C127" s="15" t="inlineStr">
         <is>
-          <t>1o: Japan</t>
+          <t>1o: Netherlands</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2o: Netherlands</t>
+          <t>2o: Tunisia</t>
         </is>
       </c>
     </row>
@@ -5099,6 +5107,7 @@
         </is>
       </c>
     </row>
+    <row r="134"/>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
@@ -5116,35 +5125,35 @@
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>2. Ivory Coast (Grupo E)</t>
+          <t>2. Scotland (Grupo C)</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>3. Egypt (Grupo G)</t>
+          <t>3. Turkey (Grupo D)</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>4. Paraguay (Grupo D)</t>
+          <t>4. Ivory Coast (Grupo E)</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="B140" t="inlineStr">
         <is>
-          <t>5. Algeria (Grupo J)</t>
+          <t>5. Japan (Grupo F)</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="B141" t="inlineStr">
         <is>
-          <t>6. Scotland (Grupo C)</t>
+          <t>6. Egypt (Grupo G)</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5167,7 @@
     <row r="143">
       <c r="B143" t="inlineStr">
         <is>
-          <t>8. Bosnia and Herzegovina (Grupo B)</t>
+          <t>8. Algeria (Grupo J)</t>
         </is>
       </c>
     </row>

</xml_diff>